<commit_message>
Actualización 2026-10-22: 1 hecho nuevo (total 31)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -238,8 +238,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH31" headerRowCount="1">
-  <autoFilter ref="A1:AH31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH32" headerRowCount="1">
+  <autoFilter ref="A1:AH32"/>
   <tableColumns count="34">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Fecha"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C13" s="4">
-        <f>COUNTA(Incidentes!A2:A31)</f>
+        <f>COUNTA(Incidentes!A2:A32)</f>
         <v/>
       </c>
     </row>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH31"/>
+  <dimension ref="A1:AH32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5424,6 +5424,157 @@
       <c r="AH31" s="6" t="inlineStr">
         <is>
           <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-031</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Valle del Cauca</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Dagua</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Corregimiento El Queremal, subestación de Policía</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>-76.69</v>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Ataque con dos artefactos explosivos lanzados desde drones contra una subestación de Policía, con civiles heridos</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Dron con explosivos</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Fuerza Pública</t>
+        </is>
+      </c>
+      <c r="M32" s="8" t="inlineStr">
+        <is>
+          <t>Presunto acto terrorista (clasificación analítica provisional)</t>
+        </is>
+      </c>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido formalmente: las autoridades señalan a la estructura Jaime Martínez como riesgo en la zona, pero indican que la responsabilidad requiere investigación</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P32" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="T32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" s="6">
+        <f>Q32+R32</f>
+        <v/>
+      </c>
+      <c r="V32" s="6">
+        <f>S32+T32</f>
+        <v/>
+      </c>
+      <c r="W32" s="8" t="inlineStr">
+        <is>
+          <t>Cuatro civiles heridos según el primer balance (esquirlas y aturdimiento); el balance podría no ser definitivo.</t>
+        </is>
+      </c>
+      <c r="X32" s="8" t="inlineStr">
+        <is>
+          <t>Las fuentes consultadas no recogen una atribución oficial de este ataque; la mención a disidencias proviene de información de prensa.</t>
+        </is>
+      </c>
+      <c r="Y32" s="8" t="inlineStr">
+        <is>
+          <t>Daños estructurales en la subestación de Policía; el segundo artefacto detonó cerca de un establecimiento comercial.</t>
+        </is>
+      </c>
+      <c r="Z32" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA32" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB32" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AC32" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD32" s="10" t="inlineStr">
+        <is>
+          <t>https://www.diariodelsur.com.co/noticias/ataque-con-explosivos-en-dagua-deja-cuatro-civiles-heridos</t>
+        </is>
+      </c>
+      <c r="AE32" s="10" t="inlineStr">
+        <is>
+          <t>https://www.semana.com/nacion/articulo/ataque-con-explosivos-aereos-contra-la-policia-en-dagua-enciende-las-alarmas-en-el-valle-del-cauca/202608/</t>
+        </is>
+      </c>
+      <c r="AF32" s="6" t="n"/>
+      <c r="AG32" s="6">
+        <f>COUNTIF(AD32:AF32,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH32" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5492,10 +5643,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE30" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF30" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD31" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD32" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE32" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId64"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5547,7 +5700,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTA(Incidentes!$A$2:$A$31)</f>
+        <f>COUNTA(Incidentes!$A$2:$A$32)</f>
         <v/>
       </c>
     </row>
@@ -5558,7 +5711,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUM(Incidentes!$U$2:$U$31)</f>
+        <f>SUM(Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
     </row>
@@ -5569,7 +5722,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUM(Incidentes!$R$2:$R$31)</f>
+        <f>SUM(Incidentes!$R$2:$R$32)</f>
         <v/>
       </c>
     </row>
@@ -5580,7 +5733,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUM(Incidentes!$Q$2:$Q$31)</f>
+        <f>SUM(Incidentes!$Q$2:$Q$32)</f>
         <v/>
       </c>
     </row>
@@ -5591,7 +5744,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUM(Incidentes!$V$2:$V$31)</f>
+        <f>SUM(Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5602,7 +5755,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUM(Incidentes!$T$2:$T$31)</f>
+        <f>SUM(Incidentes!$T$2:$T$32)</f>
         <v/>
       </c>
     </row>
@@ -5613,7 +5766,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUM(Incidentes!$S$2:$S$31)</f>
+        <f>SUM(Incidentes!$S$2:$S$32)</f>
         <v/>
       </c>
     </row>
@@ -5635,7 +5788,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$31,Incidentes!$D$2:$D$31))</f>
+        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$32,Incidentes!$D$2:$D$32))</f>
         <v/>
       </c>
     </row>
@@ -5646,7 +5799,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$31,Incidentes!$D$2:$D$31,Incidentes!$E$2:$E$31,Incidentes!$E$2:$E$31))</f>
+        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$32,Incidentes!$D$2:$D$32,Incidentes!$E$2:$E$32,Incidentes!$E$2:$E$32))</f>
         <v/>
       </c>
     </row>
@@ -5657,7 +5810,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,"ELN")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,"ELN")</f>
         <v/>
       </c>
     </row>
@@ -5668,7 +5821,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,"Disidencias FARC")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,"Disidencias FARC")</f>
         <v/>
       </c>
     </row>
@@ -5679,7 +5832,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$31,"No determinado")</f>
+        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$32,"No determinado")</f>
         <v/>
       </c>
     </row>
@@ -5690,7 +5843,7 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
     </row>
@@ -5712,7 +5865,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>COUNTIF(Incidentes!$AG$2:$AG$31,1)</f>
+        <f>COUNTIF(Incidentes!$AG$2:$AG$32,1)</f>
         <v/>
       </c>
     </row>
@@ -5723,7 +5876,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$31=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$31))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$31)))&gt;0))/B4</f>
+        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$32=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$32))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$32)))&gt;0))/B4</f>
         <v/>
       </c>
     </row>
@@ -5756,15 +5909,15 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A24)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A24)</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A24,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A24,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A24,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A24,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5775,15 +5928,15 @@
         </is>
       </c>
       <c r="B25" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A25)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A25)</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A25,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A25,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A25,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A25,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5794,15 +5947,15 @@
         </is>
       </c>
       <c r="B26" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A26)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A26)</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A26,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A26,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A26,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A26,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5813,15 +5966,15 @@
         </is>
       </c>
       <c r="B27" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A27)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A27)</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A27,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A27,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A27,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A27,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5832,15 +5985,15 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A28)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A28)</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A28,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A28,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A28,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A28,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5851,15 +6004,15 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$31,A29)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$32,A29)</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A29,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A29,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$31,A29,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$32,A29,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
     </row>
@@ -5882,7 +6035,7 @@
         </is>
       </c>
       <c r="B33" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"A")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"A")</f>
         <v/>
       </c>
     </row>
@@ -5893,7 +6046,7 @@
         </is>
       </c>
       <c r="B34" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"B")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"B")</f>
         <v/>
       </c>
     </row>
@@ -5904,7 +6057,7 @@
         </is>
       </c>
       <c r="B35" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"C")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"C")</f>
         <v/>
       </c>
     </row>
@@ -5915,7 +6068,7 @@
         </is>
       </c>
       <c r="B36" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"D")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"D")</f>
         <v/>
       </c>
     </row>
@@ -5926,7 +6079,7 @@
         </is>
       </c>
       <c r="B37" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
     </row>
@@ -5969,19 +6122,19 @@
         </is>
       </c>
       <c r="B41" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A41)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A41)</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A41,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A41,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A41,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A41,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E41" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A41,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A41,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F41" s="13">
@@ -5996,19 +6149,19 @@
         </is>
       </c>
       <c r="B42" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A42)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A42)</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A42,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A42,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A42,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A42,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E42" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A42,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A42,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F42" s="13">
@@ -6023,19 +6176,19 @@
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A43)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A43)</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A43,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A43,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A43,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A43,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A43,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A43,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F43" s="13">
@@ -6050,19 +6203,19 @@
         </is>
       </c>
       <c r="B44" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A44)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A44)</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A44,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A44,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A44,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A44,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A44,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A44,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F44" s="13">
@@ -6077,19 +6230,19 @@
         </is>
       </c>
       <c r="B45" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A45)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A45)</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A45,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A45,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A45,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A45,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A45,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A45,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F45" s="13">
@@ -6104,19 +6257,19 @@
         </is>
       </c>
       <c r="B46" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A46)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A46)</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A46,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A46,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A46,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A46,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A46,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A46,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F46" s="13">
@@ -6131,19 +6284,19 @@
         </is>
       </c>
       <c r="B47" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A47)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A47)</f>
         <v/>
       </c>
       <c r="C47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A47,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A47,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A47,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A47,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E47" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A47,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A47,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F47" s="13">
@@ -6158,19 +6311,19 @@
         </is>
       </c>
       <c r="B48" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A48)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A48)</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A48,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A48,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A48,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A48,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A48,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A48,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F48" s="13">
@@ -6185,19 +6338,19 @@
         </is>
       </c>
       <c r="B49" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A49)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A49)</f>
         <v/>
       </c>
       <c r="C49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A49,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A49,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A49,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A49,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E49" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A49,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A49,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F49" s="13">
@@ -6212,19 +6365,19 @@
         </is>
       </c>
       <c r="B50" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$31,A50)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$32,A50)</f>
         <v/>
       </c>
       <c r="C50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A50,Incidentes!$U$2:$U$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A50,Incidentes!$U$2:$U$32)</f>
         <v/>
       </c>
       <c r="D50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$31,A50,Incidentes!$V$2:$V$31)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$32,A50,Incidentes!$V$2:$V$32)</f>
         <v/>
       </c>
       <c r="E50" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$31,A50,Incidentes!$P$2:$P$31,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$32,A50,Incidentes!$P$2:$P$32,"E")</f>
         <v/>
       </c>
       <c r="F50" s="13">
@@ -6277,15 +6430,15 @@
         <v>46266</v>
       </c>
       <c r="D54" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$31,"&gt;="&amp;B54,Incidentes!$B$2:$B$31,"&lt;"&amp;C54)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
         <v/>
       </c>
       <c r="E54" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B54,Incidentes!$B$2:$B$31,"&lt;"&amp;C54)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
         <v/>
       </c>
       <c r="F54" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B54,Incidentes!$B$2:$B$31,"&lt;"&amp;C54)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
         <v/>
       </c>
     </row>
@@ -6302,15 +6455,15 @@
         <v>46296</v>
       </c>
       <c r="D55" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$31,"&gt;="&amp;B55,Incidentes!$B$2:$B$31,"&lt;"&amp;C55)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="E55" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B55,Incidentes!$B$2:$B$31,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="F55" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B55,Incidentes!$B$2:$B$31,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
         <v/>
       </c>
     </row>
@@ -6327,15 +6480,15 @@
         <v>46327</v>
       </c>
       <c r="D56" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$31,"&gt;="&amp;B56,Incidentes!$B$2:$B$31,"&lt;"&amp;C56)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="E56" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B56,Incidentes!$B$2:$B$31,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="F56" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$31,Incidentes!$B$2:$B$31,"&gt;="&amp;B56,Incidentes!$B$2:$B$31,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
         <v/>
       </c>
     </row>
@@ -6350,7 +6503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7446,76 +7599,110 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-031</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>https://www.diariodelsur.com.co/noticias/ataque-con-explosivos-en-dagua-deja-cuatro-civiles-heridos</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>diariodelsur.com.co</t>
+        </is>
+      </c>
+    </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-031</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>https://www.semana.com/nacion/articulo/ataque-con-explosivos-aereos-contra-la-policia-en-dagua-enciende-las-alarmas-en-el-valle-del-cauca/202608/</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>semana.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="14" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B69" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C67" s="14" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
         <is>
           <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
-        </is>
-      </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
-        </is>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
-        </is>
-      </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
+          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
+        </is>
+      </c>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C72" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -7586,9 +7773,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización 2026-10-24: 3 hechos nuevos (total 34)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -238,8 +238,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH32" headerRowCount="1">
-  <autoFilter ref="A1:AH32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH35" headerRowCount="1">
+  <autoFilter ref="A1:AH35"/>
   <tableColumns count="34">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Fecha"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C13" s="4">
-        <f>COUNTA(Incidentes!A2:A32)</f>
+        <f>COUNTA(Incidentes!A2:A35)</f>
         <v/>
       </c>
     </row>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5575,6 +5575,451 @@
       <c r="AH32" s="6" t="inlineStr">
         <is>
           <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-032</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Madrugada</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Casanare</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Villanueva</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Peaje San Pedro, vía Villanueva–Monterrey</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>-72.93000000000001</v>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Explosión de un presunto carro bomba en un peaje; según versiones preliminares, dos hombres dejaron un vehículo y huyeron en motocicleta</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>Vehículo con explosivos</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Infraestructura vial</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>Presunto acto terrorista (clasificación analítica provisional)</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido formalmente: la gobernación ofreció recompensa por los responsables y se investiga</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="6">
+        <f>Q33+R33</f>
+        <v/>
+      </c>
+      <c r="V33" s="6">
+        <f>S33+T33</f>
+        <v/>
+      </c>
+      <c r="W33" s="8" t="inlineStr">
+        <is>
+          <t>Cinco heridos según el último reporte consultado (el primer balance indicaba cuatro).</t>
+        </is>
+      </c>
+      <c r="X33" s="8" t="inlineStr">
+        <is>
+          <t>Las fuentes consultadas no recogen una atribución oficial; las autoridades investigan el hecho.</t>
+        </is>
+      </c>
+      <c r="Y33" s="8" t="inlineStr">
+        <is>
+          <t>Destrucción parcial de la estructura, cabinas y oficinas del peaje; tránsito suspendido.</t>
+        </is>
+      </c>
+      <c r="Z33" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA33" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB33" s="6" t="inlineStr">
+        <is>
+          <t>Cierre temporal de la vía</t>
+        </is>
+      </c>
+      <c r="AC33" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD33" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/10/23/explosion-de-un-presunto-carro-bomba-en-peaje-de-casanare-deja-cuatro-heridos-investigan-atentado/</t>
+        </is>
+      </c>
+      <c r="AE33" s="10" t="inlineStr">
+        <is>
+          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
+        </is>
+      </c>
+      <c r="AF33" s="6" t="n"/>
+      <c r="AG33" s="6">
+        <f>COUNTIF(AD33:AF33,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH33" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-033</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Cauca</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Guapi</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Sector Bonanza, zona rural</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>-77.89</v>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>Ataque con artefactos explosivos lanzados desde drones contra unidades de la Armada Nacional que adelantaban operaciones</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>Dron con explosivos</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>Fuerza Pública</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="inlineStr">
+        <is>
+          <t>Presunto acto terrorista (clasificación analítica provisional)</t>
+        </is>
+      </c>
+      <c r="N34" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido formalmente: móviles y responsables en verificación</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P34" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="U34" s="6">
+        <f>Q34+R34</f>
+        <v/>
+      </c>
+      <c r="V34" s="6">
+        <f>S34+T34</f>
+        <v/>
+      </c>
+      <c r="W34" s="8" t="inlineStr">
+        <is>
+          <t>Un infante de Marina muerto y cuatro uniformados heridos según el reporte preliminar; los heridos fueron trasladados a Cali.</t>
+        </is>
+      </c>
+      <c r="X34" s="8" t="inlineStr">
+        <is>
+          <t>La fuente consultada no recoge una atribución oficial; las autoridades adelantan verificaciones.</t>
+        </is>
+      </c>
+      <c r="Y34" s="8" t="inlineStr">
+        <is>
+          <t>Daños en la lancha utilizada por la unidad.</t>
+        </is>
+      </c>
+      <c r="Z34" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA34" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB34" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AC34" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD34" s="10" t="inlineStr">
+        <is>
+          <t>https://www.elpais.com.co/judicial/un-infante-de-marina-murio-y-cuatro-militares-resultaron-heridos-tras-ataque-con-explosivos-en-zona-rural-de-guapi-2343.html</t>
+        </is>
+      </c>
+      <c r="AE34" s="6" t="n"/>
+      <c r="AF34" s="6" t="n"/>
+      <c r="AG34" s="6">
+        <f>COUNTIF(AD34:AF34,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH34" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-034</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Madrugada</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Puerto Santander</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Vía urbana, área metropolitana de Cúcuta</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>-72.41</v>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>Detonación de un artefacto explosivo instalado al paso de una patrulla motorizada de la Policía</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>Explosivo / IED</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>Fuerza Pública</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>Presunto acto terrorista (clasificación analítica provisional)</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido formalmente: las autoridades investigan</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P35" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="6">
+        <f>Q35+R35</f>
+        <v/>
+      </c>
+      <c r="V35" s="6">
+        <f>S35+T35</f>
+        <v/>
+      </c>
+      <c r="W35" s="6" t="inlineStr">
+        <is>
+          <t>Uniformados ilesos.</t>
+        </is>
+      </c>
+      <c r="X35" s="8" t="inlineStr">
+        <is>
+          <t>La fuente consultada no recoge una atribución oficial.</t>
+        </is>
+      </c>
+      <c r="Y35" s="8" t="inlineStr">
+        <is>
+          <t>Afectación de la vía (tierra y material vegetal sobre la calzada); sin mayores daños.</t>
+        </is>
+      </c>
+      <c r="Z35" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA35" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB35" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AC35" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD35" s="10" t="inlineStr">
+        <is>
+          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
+        </is>
+      </c>
+      <c r="AE35" s="6" t="n"/>
+      <c r="AF35" s="6" t="n"/>
+      <c r="AG35" s="6">
+        <f>COUNTIF(AD35:AF35,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH35" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -5645,10 +6090,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD31" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD32" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE32" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD33" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE33" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD34" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5659,7 +6108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5700,7 +6149,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTA(Incidentes!$A$2:$A$32)</f>
+        <f>COUNTA(Incidentes!$A$2:$A$35)</f>
         <v/>
       </c>
     </row>
@@ -5711,7 +6160,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUM(Incidentes!$U$2:$U$32)</f>
+        <f>SUM(Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
     </row>
@@ -5722,7 +6171,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUM(Incidentes!$R$2:$R$32)</f>
+        <f>SUM(Incidentes!$R$2:$R$35)</f>
         <v/>
       </c>
     </row>
@@ -5733,7 +6182,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUM(Incidentes!$Q$2:$Q$32)</f>
+        <f>SUM(Incidentes!$Q$2:$Q$35)</f>
         <v/>
       </c>
     </row>
@@ -5744,7 +6193,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUM(Incidentes!$V$2:$V$32)</f>
+        <f>SUM(Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -5755,7 +6204,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUM(Incidentes!$T$2:$T$32)</f>
+        <f>SUM(Incidentes!$T$2:$T$35)</f>
         <v/>
       </c>
     </row>
@@ -5766,7 +6215,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUM(Incidentes!$S$2:$S$32)</f>
+        <f>SUM(Incidentes!$S$2:$S$35)</f>
         <v/>
       </c>
     </row>
@@ -5788,7 +6237,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$32,Incidentes!$D$2:$D$32))</f>
+        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$35,Incidentes!$D$2:$D$35))</f>
         <v/>
       </c>
     </row>
@@ -5799,7 +6248,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$32,Incidentes!$D$2:$D$32,Incidentes!$E$2:$E$32,Incidentes!$E$2:$E$32))</f>
+        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$35,Incidentes!$D$2:$D$35,Incidentes!$E$2:$E$35,Incidentes!$E$2:$E$35))</f>
         <v/>
       </c>
     </row>
@@ -5810,7 +6259,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,"ELN")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,"ELN")</f>
         <v/>
       </c>
     </row>
@@ -5821,7 +6270,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,"Disidencias FARC")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,"Disidencias FARC")</f>
         <v/>
       </c>
     </row>
@@ -5832,7 +6281,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$32,"No determinado")</f>
+        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$35,"No determinado")</f>
         <v/>
       </c>
     </row>
@@ -5843,7 +6292,7 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
     </row>
@@ -5865,7 +6314,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>COUNTIF(Incidentes!$AG$2:$AG$32,1)</f>
+        <f>COUNTIF(Incidentes!$AG$2:$AG$35,1)</f>
         <v/>
       </c>
     </row>
@@ -5876,7 +6325,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$32=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$32))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$32)))&gt;0))/B4</f>
+        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$35=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$35))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$35)))&gt;0))/B4</f>
         <v/>
       </c>
     </row>
@@ -5909,15 +6358,15 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A24)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A24)</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A24,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A24,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A24,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A24,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -5928,15 +6377,15 @@
         </is>
       </c>
       <c r="B25" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A25)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A25)</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A25,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A25,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A25,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A25,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -5947,15 +6396,15 @@
         </is>
       </c>
       <c r="B26" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A26)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A26)</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A26,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A26,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A26,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A26,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -5966,15 +6415,15 @@
         </is>
       </c>
       <c r="B27" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A27)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A27)</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A27,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A27,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A27,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A27,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -5985,15 +6434,15 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A28)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A28)</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A28,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A28,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A28,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A28,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -6004,15 +6453,15 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$32,A29)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$35,A29)</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A29,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A29,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$32,A29,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$35,A29,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
     </row>
@@ -6035,7 +6484,7 @@
         </is>
       </c>
       <c r="B33" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"A")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"A")</f>
         <v/>
       </c>
     </row>
@@ -6046,7 +6495,7 @@
         </is>
       </c>
       <c r="B34" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"B")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"B")</f>
         <v/>
       </c>
     </row>
@@ -6057,7 +6506,7 @@
         </is>
       </c>
       <c r="B35" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"C")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"C")</f>
         <v/>
       </c>
     </row>
@@ -6068,7 +6517,7 @@
         </is>
       </c>
       <c r="B36" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"D")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"D")</f>
         <v/>
       </c>
     </row>
@@ -6079,7 +6528,7 @@
         </is>
       </c>
       <c r="B37" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
     </row>
@@ -6122,19 +6571,19 @@
         </is>
       </c>
       <c r="B41" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A41)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A41)</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A41,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A41,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A41,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A41,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E41" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A41,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A41,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F41" s="13">
@@ -6145,23 +6594,23 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Cauca</t>
+          <t>Casanare</t>
         </is>
       </c>
       <c r="B42" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A42)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A42)</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A42,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A42,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A42,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A42,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E42" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A42,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A42,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F42" s="13">
@@ -6172,23 +6621,23 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Cesar</t>
+          <t>Cauca</t>
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A43)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A43)</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A43,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A43,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A43,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A43,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A43,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A43,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F43" s="13">
@@ -6199,23 +6648,23 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Chocó</t>
+          <t>Cesar</t>
         </is>
       </c>
       <c r="B44" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A44)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A44)</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A44,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A44,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A44,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A44,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A44,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A44,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F44" s="13">
@@ -6226,23 +6675,23 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Huila</t>
+          <t>Chocó</t>
         </is>
       </c>
       <c r="B45" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A45)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A45)</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A45,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A45,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A45,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A45,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A45,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A45,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F45" s="13">
@@ -6253,23 +6702,23 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>La Guajira</t>
+          <t>Huila</t>
         </is>
       </c>
       <c r="B46" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A46)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A46)</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A46,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A46,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A46,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A46,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A46,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A46,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F46" s="13">
@@ -6280,23 +6729,23 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Magdalena</t>
+          <t>La Guajira</t>
         </is>
       </c>
       <c r="B47" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A47)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A47)</f>
         <v/>
       </c>
       <c r="C47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A47,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A47,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A47,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A47,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E47" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A47,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A47,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F47" s="13">
@@ -6307,23 +6756,23 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Nariño</t>
+          <t>Magdalena</t>
         </is>
       </c>
       <c r="B48" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A48)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A48)</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A48,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A48,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A48,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A48,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A48,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A48,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F48" s="13">
@@ -6334,23 +6783,23 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Norte de Santander</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="B49" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A49)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A49)</f>
         <v/>
       </c>
       <c r="C49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A49,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A49,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A49,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A49,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E49" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A49,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A49,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F49" s="13">
@@ -6361,23 +6810,23 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Valle del Cauca</t>
+          <t>Norte de Santander</t>
         </is>
       </c>
       <c r="B50" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$32,A50)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A50)</f>
         <v/>
       </c>
       <c r="C50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A50,Incidentes!$U$2:$U$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A50,Incidentes!$U$2:$U$35)</f>
         <v/>
       </c>
       <c r="D50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$32,A50,Incidentes!$V$2:$V$32)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$35,A50,Incidentes!$V$2:$V$35)</f>
         <v/>
       </c>
       <c r="E50" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$32,A50,Incidentes!$P$2:$P$32,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A50,Incidentes!$P$2:$P$35,"E")</f>
         <v/>
       </c>
       <c r="F50" s="13">
@@ -6385,110 +6834,137 @@
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Valle del Cauca</t>
+        </is>
+      </c>
+      <c r="B51" s="6">
+        <f>COUNTIF(Incidentes!$D$2:$D$35,A51)</f>
+        <v/>
+      </c>
+      <c r="C51" s="6">
+        <f>SUMIF(Incidentes!$D$2:$D$35,A51,Incidentes!$U$2:$U$35)</f>
+        <v/>
+      </c>
+      <c r="D51" s="6">
+        <f>SUMIF(Incidentes!$D$2:$D$35,A51,Incidentes!$V$2:$V$35)</f>
+        <v/>
+      </c>
+      <c r="E51" s="6">
+        <f>COUNTIFS(Incidentes!$D$2:$D$35,A51,Incidentes!$P$2:$P$35,"E")</f>
+        <v/>
+      </c>
+      <c r="F51" s="13">
+        <f>E51/B51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>Por mes</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Desde</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Hasta (excl.)</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Incidentes</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>Fallecidos</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>Heridos</t>
         </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>agosto (desde el 7)</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C54" s="7" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D54" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
-        <v/>
-      </c>
-      <c r="E54" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
-        <v/>
-      </c>
-      <c r="F54" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B54,Incidentes!$B$2:$B$32,"&lt;"&amp;C54)</f>
-        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>septiembre</t>
+          <t>agosto (desde el 7)</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C55" s="7" t="n">
         <v>46266</v>
       </c>
-      <c r="C55" s="7" t="n">
-        <v>46296</v>
-      </c>
       <c r="D55" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="E55" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="F55" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B55,Incidentes!$B$2:$B$32,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
+          <t>septiembre</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>46266</v>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D56" s="6">
+        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <v/>
+      </c>
+      <c r="E56" s="6">
+        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <v/>
+      </c>
+      <c r="F56" s="6">
+        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
           <t>octubre</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B57" s="7" t="n">
         <v>46296</v>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C57" s="7" t="n">
         <v>46327</v>
       </c>
-      <c r="D56" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
-        <v/>
-      </c>
-      <c r="E56" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
-        <v/>
-      </c>
-      <c r="F56" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$32,Incidentes!$B$2:$B$32,"&gt;="&amp;B56,Incidentes!$B$2:$B$32,"&lt;"&amp;C56)</f>
+      <c r="D57" s="6">
+        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
+        <v/>
+      </c>
+      <c r="E57" s="6">
+        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
+        <v/>
+      </c>
+      <c r="F57" s="6">
+        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
         <v/>
       </c>
     </row>
@@ -6503,7 +6979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7633,76 +8109,144 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-032</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/10/23/explosion-de-un-presunto-carro-bomba-en-peaje-de-casanare-deja-cuatro-heridos-investigan-atentado/</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>infobae.com</t>
+        </is>
+      </c>
+    </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-032</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>noticiasrcn.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-033</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>https://www.elpais.com.co/judicial/un-infante-de-marina-murio-y-cuatro-militares-resultaron-heridos-tras-ataque-con-explosivos-en-zona-rural-de-guapi-2343.html</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>elpais.com.co</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-034</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>noticiasrcn.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B73" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C69" s="14" t="inlineStr">
+      <c r="C73" s="14" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C74" s="10" t="inlineStr">
         <is>
           <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C75" s="10" t="inlineStr">
         <is>
           <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
+      <c r="C76" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -7775,9 +8319,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización 2026-10-25: 0 hechos nuevos, 1 corrección (total 34)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5791,17 +5791,17 @@
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>No atribuido formalmente: móviles y responsables en verificación</t>
+          <t>Estructura 30 «Jhonier Toro Arenas», Bloque Occidental «Jacobo Arenas» de las disidencias de las Farc (atribución preliminar de las autoridades)</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
-          <t>No determinado</t>
+          <t>Disidencias FARC</t>
         </is>
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Q34" s="6" t="n">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="W34" s="8" t="inlineStr">
         <is>
-          <t>Un infante de Marina muerto y cuatro uniformados heridos según el reporte preliminar; los heridos fueron trasladados a Cali.</t>
+          <t>Un infante de Marina muerto y cuatro uniformados heridos (tres infantes de Marina profesionales y un suboficial), evacuados a Cali.</t>
         </is>
       </c>
       <c r="X34" s="8" t="inlineStr">
         <is>
-          <t>La fuente consultada no recoge una atribución oficial; las autoridades adelantan verificaciones.</t>
+          <t>Según información preliminar de las autoridades, el ataque lo habrían cometido integrantes de esa estructura; es una hipótesis oficial, no una conclusión confirmada.</t>
         </is>
       </c>
       <c r="Y34" s="8" t="inlineStr">
@@ -5864,7 +5864,11 @@
           <t>https://www.elpais.com.co/judicial/un-infante-de-marina-murio-y-cuatro-militares-resultaron-heridos-tras-ataque-con-explosivos-en-zona-rural-de-guapi-2343.html</t>
         </is>
       </c>
-      <c r="AE34" s="6" t="n"/>
+      <c r="AE34" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eluniversal.com.co/sucesos/2026/10/24/edwin-andres-vargas-el-infante-de-marina-que-murio-en-ataque-con-dron/</t>
+        </is>
+      </c>
       <c r="AF34" s="6" t="n"/>
       <c r="AG34" s="6">
         <f>COUNTIF(AD34:AF34,"?*")</f>
@@ -5872,7 +5876,7 @@
       </c>
       <c r="AH34" s="6" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6093,11 +6097,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD33" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE33" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD34" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId70"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6979,7 +6984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8163,90 +8168,107 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
+          <t>CO-2026-033</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eluniversal.com.co/sucesos/2026/10/24/edwin-andres-vargas-el-infante-de-marina-que-murio-en-ataque-con-dron/</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>eluniversal.com.co</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
           <t>CO-2026-034</t>
         </is>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B71" s="10" t="inlineStr">
         <is>
           <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>noticiasrcn.com</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="14" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B74" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C73" s="14" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
         <is>
           <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
-        </is>
-      </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
+          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -8323,9 +8345,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización 2026-10-26: 0 hechos nuevos (total 34); corrección Dagua
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5509,7 @@
         <v>0</v>
       </c>
       <c r="S32" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T32" s="6" t="n">
         <v>0</v>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>Cuatro civiles heridos según el primer balance (esquirlas y aturdimiento); el balance podría no ser definitivo.</t>
+          <t>Cinco civiles heridos según el balance de la Policía del Valle del Cauca (sin policías heridos).</t>
         </is>
       </c>
       <c r="X32" s="8" t="inlineStr">
@@ -5567,14 +5567,18 @@
           <t>https://www.semana.com/nacion/articulo/ataque-con-explosivos-aereos-contra-la-policia-en-dagua-enciende-las-alarmas-en-el-valle-del-cauca/202608/</t>
         </is>
       </c>
-      <c r="AF32" s="6" t="n"/>
+      <c r="AF32" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/10/14/ataque-con-drones-en-el-queremal-deja-cinco-civiles-heridos-policia-senala-a-disidencias-de-la-jaime-martinez/</t>
+        </is>
+      </c>
       <c r="AG32" s="6">
         <f>COUNTIF(AD32:AF32,"?*")</f>
         <v/>
       </c>
       <c r="AH32" s="6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6094,15 +6098,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD31" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD32" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE32" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD33" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE33" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD34" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF32" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD33" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE33" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD34" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId72"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6984,7 +6989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8117,12 +8122,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>CO-2026-032</t>
+          <t>CO-2026-031</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/10/23/explosion-de-un-presunto-carro-bomba-en-peaje-de-casanare-deja-cuatro-heridos-investigan-atentado/</t>
+          <t>https://www.infobae.com/colombia/2026/10/14/ataque-con-drones-en-el-queremal-deja-cinco-civiles-heridos-policia-senala-a-disidencias-de-la-jaime-martinez/</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -8139,29 +8144,29 @@
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
+          <t>https://www.infobae.com/colombia/2026/10/23/explosion-de-un-presunto-carro-bomba-en-peaje-de-casanare-deja-cuatro-heridos-investigan-atentado/</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>noticiasrcn.com</t>
+          <t>infobae.com</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>CO-2026-033</t>
+          <t>CO-2026-032</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>https://www.elpais.com.co/judicial/un-infante-de-marina-murio-y-cuatro-militares-resultaron-heridos-tras-ataque-con-explosivos-en-zona-rural-de-guapi-2343.html</t>
+          <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>elpais.com.co</t>
+          <t>noticiasrcn.com</t>
         </is>
       </c>
     </row>
@@ -8173,102 +8178,119 @@
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/10/24/edwin-andres-vargas-el-infante-de-marina-que-murio-en-ataque-con-dron/</t>
+          <t>https://www.elpais.com.co/judicial/un-infante-de-marina-murio-y-cuatro-militares-resultaron-heridos-tras-ataque-con-explosivos-en-zona-rural-de-guapi-2343.html</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>eluniversal.com.co</t>
+          <t>elpais.com.co</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
+          <t>CO-2026-033</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eluniversal.com.co/sucesos/2026/10/24/edwin-andres-vargas-el-infante-de-marina-que-murio-en-ataque-con-dron/</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>eluniversal.com.co</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
           <t>CO-2026-034</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B72" s="10" t="inlineStr">
         <is>
           <t>https://www.noticiasrcn.com/colombia/artefacto-explosivo-detono-al-paso-de-patrulla-en-puerto-santander-1074715</t>
         </is>
       </c>
-      <c r="C71" s="6" t="inlineStr">
+      <c r="C72" s="6" t="inlineStr">
         <is>
           <t>noticiasrcn.com</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B75" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
+      <c r="C75" s="14" t="inlineStr">
         <is>
           <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
-        </is>
-      </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
-        </is>
-      </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
+          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
+      <c r="C78" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -8346,9 +8368,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización 2026-10-29: 1 hechos nuevos (total 35)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -238,8 +238,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH35" headerRowCount="1">
-  <autoFilter ref="A1:AH35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH36" headerRowCount="1">
+  <autoFilter ref="A1:AH36"/>
   <tableColumns count="34">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Fecha"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C13" s="4">
-        <f>COUNTA(Incidentes!A2:A35)</f>
+        <f>COUNTA(Incidentes!A2:A36)</f>
         <v/>
       </c>
     </row>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH35"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6028,6 +6028,157 @@
       <c r="AH35" s="6" t="inlineStr">
         <is>
           <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-035</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>46322</v>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Mañana</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Cúcuta</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Barrio El Escobal, junto al puente internacional Francisco de Paula Santander</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>-72.5</v>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>Detonación de un artefacto explosivo detrás de la sede de la DIAN, donde se estacionan vehículos de la Policía que vigilan el puente, con civiles y policías heridos</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>Explosivo / IED</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>Fuerza Pública</t>
+        </is>
+      </c>
+      <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>Presunto acto terrorista (clasificación analítica provisional)</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido formalmente: las autoridades investigan y la Gobernación y la Alcaldía ofrecen recompensa</t>
+        </is>
+      </c>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="T36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U36" s="6">
+        <f>Q36+R36</f>
+        <v/>
+      </c>
+      <c r="V36" s="6">
+        <f>S36+T36</f>
+        <v/>
+      </c>
+      <c r="W36" s="8" t="inlineStr">
+        <is>
+          <t>Seis heridos (cuatro civiles y dos policías) según el último balance consultado.</t>
+        </is>
+      </c>
+      <c r="X36" s="8" t="inlineStr">
+        <is>
+          <t>Las fuentes consultadas no recogen una atribución oficial; ningún grupo se ha adjudicado el hecho.</t>
+        </is>
+      </c>
+      <c r="Y36" s="6" t="inlineStr">
+        <is>
+          <t>No informados con precisión.</t>
+        </is>
+      </c>
+      <c r="Z36" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA36" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB36" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AC36" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD36" s="10" t="inlineStr">
+        <is>
+          <t>https://www.diariodelsur.com.co/noticias/atentado-en-cucuta-deja-seis-personas-heridas-cerca-de-la-frontera</t>
+        </is>
+      </c>
+      <c r="AE36" s="10" t="inlineStr">
+        <is>
+          <t>https://www.ntn24.com/noticias-actualidad/atentado-en-cucuta-deja-varios-heridos-horas-despues-del-asesinato-de-miguel-castellanos-esto-se-sabe-661670</t>
+        </is>
+      </c>
+      <c r="AF36" s="6" t="n"/>
+      <c r="AG36" s="6">
+        <f>COUNTIF(AD36:AF36,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH36" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -6104,10 +6255,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD34" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE36" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId72"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId74"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6159,7 +6312,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTA(Incidentes!$A$2:$A$35)</f>
+        <f>COUNTA(Incidentes!$A$2:$A$36)</f>
         <v/>
       </c>
     </row>
@@ -6170,7 +6323,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUM(Incidentes!$U$2:$U$35)</f>
+        <f>SUM(Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
     </row>
@@ -6181,7 +6334,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUM(Incidentes!$R$2:$R$35)</f>
+        <f>SUM(Incidentes!$R$2:$R$36)</f>
         <v/>
       </c>
     </row>
@@ -6192,7 +6345,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUM(Incidentes!$Q$2:$Q$35)</f>
+        <f>SUM(Incidentes!$Q$2:$Q$36)</f>
         <v/>
       </c>
     </row>
@@ -6203,7 +6356,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUM(Incidentes!$V$2:$V$35)</f>
+        <f>SUM(Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6214,7 +6367,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUM(Incidentes!$T$2:$T$35)</f>
+        <f>SUM(Incidentes!$T$2:$T$36)</f>
         <v/>
       </c>
     </row>
@@ -6225,7 +6378,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUM(Incidentes!$S$2:$S$35)</f>
+        <f>SUM(Incidentes!$S$2:$S$36)</f>
         <v/>
       </c>
     </row>
@@ -6247,7 +6400,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$35,Incidentes!$D$2:$D$35))</f>
+        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$36,Incidentes!$D$2:$D$36))</f>
         <v/>
       </c>
     </row>
@@ -6258,7 +6411,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$35,Incidentes!$D$2:$D$35,Incidentes!$E$2:$E$35,Incidentes!$E$2:$E$35))</f>
+        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$36,Incidentes!$D$2:$D$36,Incidentes!$E$2:$E$36,Incidentes!$E$2:$E$36))</f>
         <v/>
       </c>
     </row>
@@ -6269,7 +6422,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,"ELN")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,"ELN")</f>
         <v/>
       </c>
     </row>
@@ -6280,7 +6433,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,"Disidencias FARC")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,"Disidencias FARC")</f>
         <v/>
       </c>
     </row>
@@ -6291,7 +6444,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$35,"No determinado")</f>
+        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$36,"No determinado")</f>
         <v/>
       </c>
     </row>
@@ -6302,7 +6455,7 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
     </row>
@@ -6324,7 +6477,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>COUNTIF(Incidentes!$AG$2:$AG$35,1)</f>
+        <f>COUNTIF(Incidentes!$AG$2:$AG$36,1)</f>
         <v/>
       </c>
     </row>
@@ -6335,7 +6488,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$35=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$35))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$35)))&gt;0))/B4</f>
+        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$36=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$36))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$36)))&gt;0))/B4</f>
         <v/>
       </c>
     </row>
@@ -6368,15 +6521,15 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A24)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A24)</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A24,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A24,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A24,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A24,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6387,15 +6540,15 @@
         </is>
       </c>
       <c r="B25" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A25)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A25)</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A25,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A25,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A25,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A25,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6406,15 +6559,15 @@
         </is>
       </c>
       <c r="B26" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A26)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A26)</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A26,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A26,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A26,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A26,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6425,15 +6578,15 @@
         </is>
       </c>
       <c r="B27" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A27)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A27)</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A27,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A27,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A27,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A27,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6444,15 +6597,15 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A28)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A28)</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A28,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A28,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A28,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A28,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6463,15 +6616,15 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$35,A29)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$36,A29)</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A29,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A29,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$35,A29,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$36,A29,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
     </row>
@@ -6494,7 +6647,7 @@
         </is>
       </c>
       <c r="B33" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"A")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"A")</f>
         <v/>
       </c>
     </row>
@@ -6505,7 +6658,7 @@
         </is>
       </c>
       <c r="B34" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"B")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"B")</f>
         <v/>
       </c>
     </row>
@@ -6516,7 +6669,7 @@
         </is>
       </c>
       <c r="B35" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"C")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"C")</f>
         <v/>
       </c>
     </row>
@@ -6527,7 +6680,7 @@
         </is>
       </c>
       <c r="B36" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"D")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"D")</f>
         <v/>
       </c>
     </row>
@@ -6538,7 +6691,7 @@
         </is>
       </c>
       <c r="B37" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
     </row>
@@ -6581,19 +6734,19 @@
         </is>
       </c>
       <c r="B41" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A41)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A41)</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A41,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A41,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A41,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A41,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E41" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A41,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A41,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F41" s="13">
@@ -6608,19 +6761,19 @@
         </is>
       </c>
       <c r="B42" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A42)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A42)</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A42,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A42,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A42,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A42,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E42" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A42,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A42,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F42" s="13">
@@ -6635,19 +6788,19 @@
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A43)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A43)</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A43,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A43,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A43,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A43,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A43,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A43,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F43" s="13">
@@ -6662,19 +6815,19 @@
         </is>
       </c>
       <c r="B44" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A44)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A44)</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A44,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A44,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A44,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A44,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A44,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A44,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F44" s="13">
@@ -6689,19 +6842,19 @@
         </is>
       </c>
       <c r="B45" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A45)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A45)</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A45,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A45,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A45,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A45,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A45,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A45,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F45" s="13">
@@ -6716,19 +6869,19 @@
         </is>
       </c>
       <c r="B46" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A46)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A46)</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A46,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A46,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A46,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A46,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A46,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A46,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F46" s="13">
@@ -6743,19 +6896,19 @@
         </is>
       </c>
       <c r="B47" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A47)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A47)</f>
         <v/>
       </c>
       <c r="C47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A47,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A47,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A47,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A47,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E47" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A47,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A47,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F47" s="13">
@@ -6770,19 +6923,19 @@
         </is>
       </c>
       <c r="B48" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A48)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A48)</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A48,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A48,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A48,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A48,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A48,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A48,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F48" s="13">
@@ -6797,19 +6950,19 @@
         </is>
       </c>
       <c r="B49" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A49)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A49)</f>
         <v/>
       </c>
       <c r="C49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A49,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A49,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A49,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A49,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E49" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A49,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A49,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F49" s="13">
@@ -6824,19 +6977,19 @@
         </is>
       </c>
       <c r="B50" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A50)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A50)</f>
         <v/>
       </c>
       <c r="C50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A50,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A50,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A50,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A50,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E50" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A50,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A50,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F50" s="13">
@@ -6851,19 +7004,19 @@
         </is>
       </c>
       <c r="B51" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$35,A51)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$36,A51)</f>
         <v/>
       </c>
       <c r="C51" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A51,Incidentes!$U$2:$U$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A51,Incidentes!$U$2:$U$36)</f>
         <v/>
       </c>
       <c r="D51" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$35,A51,Incidentes!$V$2:$V$35)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$36,A51,Incidentes!$V$2:$V$36)</f>
         <v/>
       </c>
       <c r="E51" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$35,A51,Incidentes!$P$2:$P$35,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$36,A51,Incidentes!$P$2:$P$36,"E")</f>
         <v/>
       </c>
       <c r="F51" s="13">
@@ -6916,15 +7069,15 @@
         <v>46266</v>
       </c>
       <c r="D55" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="E55" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="F55" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B55,Incidentes!$B$2:$B$35,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
         <v/>
       </c>
     </row>
@@ -6941,15 +7094,15 @@
         <v>46296</v>
       </c>
       <c r="D56" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="E56" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="F56" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B56,Incidentes!$B$2:$B$35,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
         <v/>
       </c>
     </row>
@@ -6966,15 +7119,15 @@
         <v>46327</v>
       </c>
       <c r="D57" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
         <v/>
       </c>
       <c r="E57" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
         <v/>
       </c>
       <c r="F57" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$35,Incidentes!$B$2:$B$35,"&gt;="&amp;B57,Incidentes!$B$2:$B$35,"&lt;"&amp;C57)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
         <v/>
       </c>
     </row>
@@ -6989,7 +7142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8221,76 +8374,110 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-035</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>https://www.diariodelsur.com.co/noticias/atentado-en-cucuta-deja-seis-personas-heridas-cerca-de-la-frontera</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>diariodelsur.com.co</t>
+        </is>
+      </c>
+    </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-035</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>https://www.ntn24.com/noticias-actualidad/atentado-en-cucuta-deja-varios-heridos-horas-despues-del-asesinato-de-miguel-castellanos-esto-se-sabe-661670</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>ntn24.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C75" s="14" t="inlineStr">
+      <c r="C77" s="14" t="inlineStr">
         <is>
           <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
-        </is>
-      </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
-        </is>
-      </c>
-      <c r="B77" s="8" t="inlineStr">
-        <is>
-          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
-        </is>
-      </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
+          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -8369,9 +8556,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8383,7 +8572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9011,6 +9200,33 @@
       <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Fecha no verificable en la nota consultada; podría corresponder a hechos de junio en Suárez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Cúcuta</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Homicidio de un precandidato a la Alcaldía (baleado en la noche)</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Sin vínculo documentado con terrorismo o violencia armada organizada; autoría no establecida.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización 2026-10-30: 1 hechos nuevos (total 36)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
+++ b/dist/Observatorio_Violencia_Armada_Colombia_2026.xlsx
@@ -238,8 +238,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH36" headerRowCount="1">
-  <autoFilter ref="A1:AH36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Incidentes" displayName="Incidentes" ref="A1:AH37" headerRowCount="1">
+  <autoFilter ref="A1:AH37"/>
   <tableColumns count="34">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Fecha"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C13" s="4">
-        <f>COUNTA(Incidentes!A2:A36)</f>
+        <f>COUNTA(Incidentes!A2:A37)</f>
         <v/>
       </c>
     </row>
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH36"/>
+  <dimension ref="A1:AH37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6179,6 +6179,157 @@
       <c r="AH36" s="6" t="inlineStr">
         <is>
           <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-036</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>46324</v>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Mañana</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>El Tarra</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Sector Kilómetro 90, zona rural</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>-73.09999999999999</v>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Municipal aproximada</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Ataque con un dron cargado con explosivos que dejó civiles heridos, en medio de enfrentamientos entre el ELN y el Frente 33 de las disidencias</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>Dron con explosivos</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Población civil</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>Incierto — autoría y finalidad no establecidas</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>No atribuido: las fuentes consultadas no atribuyen el ataque a ningún grupo</t>
+        </is>
+      </c>
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>No determinado</t>
+        </is>
+      </c>
+      <c r="P37" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="Q37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" s="6">
+        <f>Q37+R37</f>
+        <v/>
+      </c>
+      <c r="V37" s="6">
+        <f>S37+T37</f>
+        <v/>
+      </c>
+      <c r="W37" s="8" t="inlineStr">
+        <is>
+          <t>Tres civiles heridos (un adulto mayor y dos jóvenes), según información preliminar.</t>
+        </is>
+      </c>
+      <c r="X37" s="8" t="inlineStr">
+        <is>
+          <t>Las fuentes consultadas no recogen una atribución oficial del ataque con dron; el Ejército halló, a pocos kilómetros una bandera con explosivos alusiva al ELN, sin vincularla formalmente con este hecho.</t>
+        </is>
+      </c>
+      <c r="Y37" s="6" t="inlineStr">
+        <is>
+          <t>No informados.</t>
+        </is>
+      </c>
+      <c r="Z37" s="6" t="inlineStr">
+        <is>
+          <t>No cuantificado</t>
+        </is>
+      </c>
+      <c r="AA37" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AB37" s="6" t="inlineStr">
+        <is>
+          <t>No documentado</t>
+        </is>
+      </c>
+      <c r="AC37" s="6" t="inlineStr">
+        <is>
+          <t>Preliminar</t>
+        </is>
+      </c>
+      <c r="AD37" s="10" t="inlineStr">
+        <is>
+          <t>https://360radio.com.co/dron-explisivos-tarra-catatumbo235911-2/235911/</t>
+        </is>
+      </c>
+      <c r="AE37" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eluniversal.com.co/colombia/2026/10/29/norte-de-santander-frustran-atentado-cerca-del-sitio-donde-exploto-un-dron/</t>
+        </is>
+      </c>
+      <c r="AF37" s="6" t="n"/>
+      <c r="AG37" s="6">
+        <f>COUNTIF(AD37:AF37,"?*")</f>
+        <v/>
+      </c>
+      <c r="AH37" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -6257,10 +6408,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE36" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD37" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId74"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId76"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6312,7 +6465,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTA(Incidentes!$A$2:$A$36)</f>
+        <f>COUNTA(Incidentes!$A$2:$A$37)</f>
         <v/>
       </c>
     </row>
@@ -6323,7 +6476,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUM(Incidentes!$U$2:$U$36)</f>
+        <f>SUM(Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
     </row>
@@ -6334,7 +6487,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUM(Incidentes!$R$2:$R$36)</f>
+        <f>SUM(Incidentes!$R$2:$R$37)</f>
         <v/>
       </c>
     </row>
@@ -6345,7 +6498,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUM(Incidentes!$Q$2:$Q$36)</f>
+        <f>SUM(Incidentes!$Q$2:$Q$37)</f>
         <v/>
       </c>
     </row>
@@ -6356,7 +6509,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUM(Incidentes!$V$2:$V$36)</f>
+        <f>SUM(Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6367,7 +6520,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUM(Incidentes!$T$2:$T$36)</f>
+        <f>SUM(Incidentes!$T$2:$T$37)</f>
         <v/>
       </c>
     </row>
@@ -6378,7 +6531,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUM(Incidentes!$S$2:$S$36)</f>
+        <f>SUM(Incidentes!$S$2:$S$37)</f>
         <v/>
       </c>
     </row>
@@ -6400,7 +6553,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$36,Incidentes!$D$2:$D$36))</f>
+        <f>SUMPRODUCT(1/COUNTIF(Incidentes!$D$2:$D$37,Incidentes!$D$2:$D$37))</f>
         <v/>
       </c>
     </row>
@@ -6411,7 +6564,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$36,Incidentes!$D$2:$D$36,Incidentes!$E$2:$E$36,Incidentes!$E$2:$E$36))</f>
+        <f>SUMPRODUCT(1/COUNTIFS(Incidentes!$D$2:$D$37,Incidentes!$D$2:$D$37,Incidentes!$E$2:$E$37,Incidentes!$E$2:$E$37))</f>
         <v/>
       </c>
     </row>
@@ -6422,7 +6575,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,"ELN")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,"ELN")</f>
         <v/>
       </c>
     </row>
@@ -6433,7 +6586,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,"Disidencias FARC")</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,"Disidencias FARC")</f>
         <v/>
       </c>
     </row>
@@ -6444,7 +6597,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$36,"No determinado")</f>
+        <f>B4-B14-B15-COUNTIF(Incidentes!$O$2:$O$37,"No determinado")</f>
         <v/>
       </c>
     </row>
@@ -6455,7 +6608,7 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
     </row>
@@ -6477,7 +6630,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>COUNTIF(Incidentes!$AG$2:$AG$36,1)</f>
+        <f>COUNTIF(Incidentes!$AG$2:$AG$37,1)</f>
         <v/>
       </c>
     </row>
@@ -6488,7 +6641,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$36=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$36))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$36)))&gt;0))/B4</f>
+        <f>SUMPRODUCT(--(((Incidentes!$AG$2:$AG$37=1)+ISNUMBER(SEARCH("Preliminar",Incidentes!$AC$2:$AC$37))+ISNUMBER(SEARCH("investigación",Incidentes!$AC$2:$AC$37)))&gt;0))/B4</f>
         <v/>
       </c>
     </row>
@@ -6521,15 +6674,15 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A24)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A24)</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A24,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A24,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A24,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A24,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6540,15 +6693,15 @@
         </is>
       </c>
       <c r="B25" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A25)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A25)</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A25,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A25,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A25,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A25,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6559,15 +6712,15 @@
         </is>
       </c>
       <c r="B26" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A26)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A26)</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A26,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A26,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A26,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A26,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6578,15 +6731,15 @@
         </is>
       </c>
       <c r="B27" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A27)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A27)</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A27,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A27,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A27,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A27,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6597,15 +6750,15 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A28)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A28)</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A28,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A28,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A28,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A28,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6616,15 +6769,15 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>COUNTIF(Incidentes!$O$2:$O$36,A29)</f>
+        <f>COUNTIF(Incidentes!$O$2:$O$37,A29)</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A29,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A29,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>SUMIF(Incidentes!$O$2:$O$36,A29,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$O$2:$O$37,A29,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
     </row>
@@ -6647,7 +6800,7 @@
         </is>
       </c>
       <c r="B33" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"A")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"A")</f>
         <v/>
       </c>
     </row>
@@ -6658,7 +6811,7 @@
         </is>
       </c>
       <c r="B34" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"B")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"B")</f>
         <v/>
       </c>
     </row>
@@ -6669,7 +6822,7 @@
         </is>
       </c>
       <c r="B35" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"C")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"C")</f>
         <v/>
       </c>
     </row>
@@ -6680,7 +6833,7 @@
         </is>
       </c>
       <c r="B36" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"D")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"D")</f>
         <v/>
       </c>
     </row>
@@ -6691,7 +6844,7 @@
         </is>
       </c>
       <c r="B37" s="6">
-        <f>COUNTIF(Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIF(Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
     </row>
@@ -6734,19 +6887,19 @@
         </is>
       </c>
       <c r="B41" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A41)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A41)</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A41,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A41,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D41" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A41,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A41,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E41" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A41,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A41,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F41" s="13">
@@ -6761,19 +6914,19 @@
         </is>
       </c>
       <c r="B42" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A42)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A42)</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A42,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A42,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D42" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A42,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A42,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E42" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A42,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A42,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F42" s="13">
@@ -6788,19 +6941,19 @@
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A43)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A43)</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A43,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A43,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A43,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A43,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A43,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A43,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F43" s="13">
@@ -6815,19 +6968,19 @@
         </is>
       </c>
       <c r="B44" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A44)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A44)</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A44,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A44,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A44,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A44,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A44,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A44,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F44" s="13">
@@ -6842,19 +6995,19 @@
         </is>
       </c>
       <c r="B45" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A45)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A45)</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A45,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A45,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D45" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A45,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A45,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A45,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A45,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F45" s="13">
@@ -6869,19 +7022,19 @@
         </is>
       </c>
       <c r="B46" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A46)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A46)</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A46,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A46,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D46" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A46,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A46,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A46,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A46,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F46" s="13">
@@ -6896,19 +7049,19 @@
         </is>
       </c>
       <c r="B47" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A47)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A47)</f>
         <v/>
       </c>
       <c r="C47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A47,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A47,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D47" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A47,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A47,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E47" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A47,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A47,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F47" s="13">
@@ -6923,19 +7076,19 @@
         </is>
       </c>
       <c r="B48" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A48)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A48)</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A48,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A48,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D48" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A48,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A48,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A48,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A48,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F48" s="13">
@@ -6950,19 +7103,19 @@
         </is>
       </c>
       <c r="B49" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A49)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A49)</f>
         <v/>
       </c>
       <c r="C49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A49,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A49,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D49" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A49,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A49,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E49" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A49,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A49,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F49" s="13">
@@ -6977,19 +7130,19 @@
         </is>
       </c>
       <c r="B50" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A50)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A50)</f>
         <v/>
       </c>
       <c r="C50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A50,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A50,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D50" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A50,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A50,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E50" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A50,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A50,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F50" s="13">
@@ -7004,19 +7157,19 @@
         </is>
       </c>
       <c r="B51" s="6">
-        <f>COUNTIF(Incidentes!$D$2:$D$36,A51)</f>
+        <f>COUNTIF(Incidentes!$D$2:$D$37,A51)</f>
         <v/>
       </c>
       <c r="C51" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A51,Incidentes!$U$2:$U$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A51,Incidentes!$U$2:$U$37)</f>
         <v/>
       </c>
       <c r="D51" s="6">
-        <f>SUMIF(Incidentes!$D$2:$D$36,A51,Incidentes!$V$2:$V$36)</f>
+        <f>SUMIF(Incidentes!$D$2:$D$37,A51,Incidentes!$V$2:$V$37)</f>
         <v/>
       </c>
       <c r="E51" s="6">
-        <f>COUNTIFS(Incidentes!$D$2:$D$36,A51,Incidentes!$P$2:$P$36,"E")</f>
+        <f>COUNTIFS(Incidentes!$D$2:$D$37,A51,Incidentes!$P$2:$P$37,"E")</f>
         <v/>
       </c>
       <c r="F51" s="13">
@@ -7069,15 +7222,15 @@
         <v>46266</v>
       </c>
       <c r="D55" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$37,"&gt;="&amp;B55,Incidentes!$B$2:$B$37,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="E55" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B55,Incidentes!$B$2:$B$37,"&lt;"&amp;C55)</f>
         <v/>
       </c>
       <c r="F55" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B55,Incidentes!$B$2:$B$36,"&lt;"&amp;C55)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B55,Incidentes!$B$2:$B$37,"&lt;"&amp;C55)</f>
         <v/>
       </c>
     </row>
@@ -7094,15 +7247,15 @@
         <v>46296</v>
       </c>
       <c r="D56" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$37,"&gt;="&amp;B56,Incidentes!$B$2:$B$37,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="E56" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B56,Incidentes!$B$2:$B$37,"&lt;"&amp;C56)</f>
         <v/>
       </c>
       <c r="F56" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B56,Incidentes!$B$2:$B$36,"&lt;"&amp;C56)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B56,Incidentes!$B$2:$B$37,"&lt;"&amp;C56)</f>
         <v/>
       </c>
     </row>
@@ -7119,15 +7272,15 @@
         <v>46327</v>
       </c>
       <c r="D57" s="6">
-        <f>COUNTIFS(Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
+        <f>COUNTIFS(Incidentes!$B$2:$B$37,"&gt;="&amp;B57,Incidentes!$B$2:$B$37,"&lt;"&amp;C57)</f>
         <v/>
       </c>
       <c r="E57" s="6">
-        <f>SUMIFS(Incidentes!$U$2:$U$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
+        <f>SUMIFS(Incidentes!$U$2:$U$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B57,Incidentes!$B$2:$B$37,"&lt;"&amp;C57)</f>
         <v/>
       </c>
       <c r="F57" s="6">
-        <f>SUMIFS(Incidentes!$V$2:$V$36,Incidentes!$B$2:$B$36,"&gt;="&amp;B57,Incidentes!$B$2:$B$36,"&lt;"&amp;C57)</f>
+        <f>SUMIFS(Incidentes!$V$2:$V$37,Incidentes!$B$2:$B$37,"&gt;="&amp;B57,Incidentes!$B$2:$B$37,"&lt;"&amp;C57)</f>
         <v/>
       </c>
     </row>
@@ -7142,7 +7295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8408,76 +8561,110 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-036</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>https://360radio.com.co/dron-explisivos-tarra-catatumbo235911-2/235911/</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>360radio.com.co</t>
+        </is>
+      </c>
+    </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>CO-2026-036</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eluniversal.com.co/colombia/2026/10/29/norte-de-santander-frustran-atentado-cerca-del-sitio-donde-exploto-un-dron/</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>eluniversal.com.co</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>Contexto agregado (no se suma a la base)</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="14" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B79" s="14" t="inlineStr">
         <is>
           <t>Cifra agregada descrita</t>
         </is>
       </c>
-      <c r="C77" s="14" t="inlineStr">
+      <c r="C79" s="14" t="inlineStr">
         <is>
           <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
-        </is>
-      </c>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
-        </is>
-      </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="8" t="inlineStr">
-        <is>
-          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
-        </is>
-      </c>
-      <c r="B79" s="8" t="inlineStr">
-        <is>
-          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
-        </is>
-      </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
+          <t>Balance de la fuerza pública citado por El Tiempo (vía Teleamazonas)</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>292 ataques con drones en 2026 con corte al 15-sep-2026, frente a 277 en todo 2025. Fuente secundaria; no se verificó el balance original.</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>https://www.teleamazonas.com/actualidad/noticias/internacional/cronologia-violencia-colombia-atentados-seguridad-129149/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>El Tiempo, citado por Infobae (2-sep-2026)</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Al menos 204 atentados con explosivos en 2026: 174 hasta el 30-jul y al menos 30 en agosto; al menos 75 atribuidos al ELN.</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/09/02/atentados-con-explosivos-en-colombia-llegan-a-204-en-2026-tras-carro-bomba-en-los-patios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
           <t>Defensoría del Pueblo, citada por Al Jazeera (18-sep-2026)</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B82" s="8" t="inlineStr">
         <is>
           <t>Los ataques con drones contra la Fuerza Pública aumentaron 146 % entre enero y mayo de 2026 frente al mismo periodo de 2025.</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
         <is>
           <t>https://www.aljazeera.com/amp/news/2026/9/18/drone-attacks-by-colombian-armed-groups-more-than-double-in-early-2026</t>
         </is>
@@ -8558,9 +8745,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8572,7 +8761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9227,6 +9416,33 @@
       <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Sin vínculo documentado con terrorismo o violencia armada organizada; autoría no establecida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>El Tarra</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Bandera con explosivos hallada y destruida por el Ejército en la vía rural (atentado frustrado)</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Atentado frustrado sin detonación.</t>
         </is>
       </c>
     </row>

</xml_diff>